<commit_message>
2026 Unlimited. Timetable Change Jul 2026.
</commit_message>
<xml_diff>
--- a/設計データ他/設計・設定.xlsx
+++ b/設計データ他/設計・設定.xlsx
@@ -160,25 +160,25 @@
     <t xml:space="preserve">"spans":[], "days":["2026/1/1"]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2026/1/4-2026/3/8", "2026/6/1-2026/7/17", "2026/9/1-2026/10/9", "2026/11/9-2026/12/20"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2026/1/4-2026/3/8", "2026/6/1-2026/8/7", "2026/8/17-2026/12/30"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2026/3/9-2026/5/31", "2026/7/18-2026/8/31", "2026/10/10-2026/11/8", "2026/12/21-2026/12/30"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2026/3/9-2026/5/31", "2026/8/8-2026/8/16"], "days":[]</t>
   </si>
   <si>
     <t xml:space="preserve">"spans":["2025/12/31-2026/1/3"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2026/1/4-2026/2/28", "2026/6/1-2026/7/17", "2026/11/9-2026/12/20"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/10/10-2026/12/30"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2026/4/1-2026/5/31", "2026/7/18-2026/8/31", "2026/11/1-2026/11/8", "2026/12/21-2026/12/30"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2026/4/1-2026/5/31", "2026/8/8-2026/8/16"], "days":[]</t>
   </si>
   <si>
     <t xml:space="preserve">"spans":["2026/3/1-2026/3/8", "2026/9/1-2026/10/9"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2026/3/9-2026/3/31", "2026/10/10-2026/10/31"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2026/3/9-2026/3/31"], "days":[]</t>
   </si>
   <si>
     <t xml:space="preserve">"spans":["2025/1/1-2025/3/9", "2025/6/17-2025/7/18", "2025/9/1-2025/9/30", "2025/11/4-2025/12/20"], "days":[]</t>
@@ -281,7 +281,7 @@
     <numFmt numFmtId="166" formatCode="0_ "/>
     <numFmt numFmtId="167" formatCode="h:mm"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -371,6 +371,13 @@
     <font>
       <sz val="24"/>
       <color theme="1"/>
+      <name val="Noto Serif JP"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="24"/>
+      <color rgb="FF000000"/>
       <name val="Noto Serif JP"/>
       <family val="2"/>
       <charset val="128"/>
@@ -491,143 +498,143 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -644,7 +651,7 @@
   <dxfs count="8">
     <dxf>
       <font>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill>
@@ -659,7 +666,7 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill>
@@ -674,7 +681,7 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill>
@@ -689,7 +696,7 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill>
@@ -777,9 +784,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>696960</xdr:colOff>
+      <xdr:colOff>696600</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>81720</xdr:rowOff>
+      <xdr:rowOff>81360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -789,7 +796,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2207880" y="5153040"/>
-          <a:ext cx="8536680" cy="3200040"/>
+          <a:ext cx="8536320" cy="3199680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -799,9 +806,7 @@
         </a:solidFill>
         <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="ffffff">
-              <a:shade val="50000"/>
-            </a:srgbClr>
+            <a:srgbClr val="bcbcbc"/>
           </a:solidFill>
           <a:round/>
         </a:ln>
@@ -954,9 +959,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>66240</xdr:colOff>
+      <xdr:colOff>65880</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>167400</xdr:rowOff>
+      <xdr:rowOff>167040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -966,7 +971,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="637920"/>
-          <a:ext cx="8603280" cy="628560"/>
+          <a:ext cx="8602920" cy="628200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -978,9 +983,7 @@
         </a:solidFill>
         <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="ffffff">
-              <a:shade val="50000"/>
-            </a:srgbClr>
+            <a:srgbClr val="bcbcbc"/>
           </a:solidFill>
           <a:round/>
         </a:ln>
@@ -1058,9 +1061,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>696960</xdr:colOff>
+      <xdr:colOff>696600</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>81720</xdr:rowOff>
+      <xdr:rowOff>81360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1070,7 +1073,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2207880" y="5153040"/>
-          <a:ext cx="8536680" cy="3200040"/>
+          <a:ext cx="8536320" cy="3199680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1080,9 +1083,7 @@
         </a:solidFill>
         <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="ffffff">
-              <a:shade val="50000"/>
-            </a:srgbClr>
+            <a:srgbClr val="bcbcbc"/>
           </a:solidFill>
           <a:round/>
         </a:ln>
@@ -1263,9 +1264,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>1866240</xdr:colOff>
+      <xdr:colOff>1865880</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>81720</xdr:rowOff>
+      <xdr:rowOff>81360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1275,7 +1276,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2067120" y="4695840"/>
-          <a:ext cx="9955440" cy="2742840"/>
+          <a:ext cx="9955080" cy="2742480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1285,9 +1286,7 @@
         </a:solidFill>
         <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="ffffff">
-              <a:shade val="50000"/>
-            </a:srgbClr>
+            <a:srgbClr val="bcbcbc"/>
           </a:solidFill>
           <a:round/>
         </a:ln>
@@ -1468,9 +1467,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>1866240</xdr:colOff>
+      <xdr:colOff>1865880</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>81720</xdr:rowOff>
+      <xdr:rowOff>81360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1480,7 +1479,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2067120" y="4695840"/>
-          <a:ext cx="9955440" cy="2057040"/>
+          <a:ext cx="9955080" cy="2056680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1490,9 +1489,7 @@
         </a:solidFill>
         <a:ln w="9525">
           <a:solidFill>
-            <a:srgbClr val="ffffff">
-              <a:shade val="50000"/>
-            </a:srgbClr>
+            <a:srgbClr val="bcbcbc"/>
           </a:solidFill>
           <a:round/>
         </a:ln>
@@ -12487,12 +12484,12 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{963D94AF-7A4A-403E-98FC-431928813FA0}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{E2BAB997-E02C-43CF-A2D0-2D3DEC14A97A}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
               <font>
-                <color rgb="00FFFFFF"/>
+                <color rgb="FFFFFFFF"/>
               </font>
               <fill>
                 <patternFill>
@@ -12501,7 +12498,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{1844F4C8-4B27-4434-B896-BC4E3037259D}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{DA90B542-3FD6-49C0-B339-2F7653A86F78}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>
@@ -13504,7 +13501,7 @@
       </c>
       <c r="CM4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; CJ4 &amp; """, " &amp; CK2 &amp; CL3 &amp; ", ""info"":""" &amp; CJ2 &amp; """, ""data"":["</f>
-        <v>{"ship":"フェリーどうぜん", "spans":["2026/1/4-2026/3/8", "2026/6/1-2026/7/17", "2026/9/1-2026/10/9", "2026/11/9-2026/12/20"], "days":[], "info":"2026通常、汽船２隻", "data":[</v>
+        <v>{"ship":"フェリーどうぜん", "spans":["2026/1/4-2026/3/8", "2026/6/1-2026/8/7", "2026/8/17-2026/12/30"], "days":[], "info":"2026通常、汽船２隻", "data":[</v>
       </c>
       <c r="CO4" s="8" t="s">
         <v>25</v>
@@ -13517,7 +13514,7 @@
       </c>
       <c r="CR4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; CO4 &amp; """, " &amp; CP2 &amp; CQ3 &amp; ", ""info"":""" &amp; CO2 &amp; """, ""data"":["</f>
-        <v>{"ship":"フェリーどうぜん", "spans":["2026/3/9-2026/5/31", "2026/7/18-2026/8/31", "2026/10/10-2026/11/8", "2026/12/21-2026/12/30"], "days":[], "info":"2026通常、汽船３隻", "data":[</v>
+        <v>{"ship":"フェリーどうぜん", "spans":["2026/3/9-2026/5/31", "2026/8/8-2026/8/16"], "days":[], "info":"2026通常、汽船３隻", "data":[</v>
       </c>
       <c r="CU4" s="8" t="s">
         <v>26</v>
@@ -13543,7 +13540,7 @@
       </c>
       <c r="DC4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; CZ4 &amp; """, " &amp; DA2 &amp; DB3 &amp; ", ""info"":""" &amp; CZ2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/7/17", "2026/11/9-2026/12/20"], "days":[], "info":"2026通常、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/10/10-2026/12/30"], "days":[], "info":"2026通常、汽船２隻", "data":[</v>
       </c>
       <c r="DE4" s="8" t="s">
         <v>26</v>
@@ -13556,7 +13553,7 @@
       </c>
       <c r="DH4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DE4 &amp; """, " &amp; DF2 &amp; DG3 &amp; ", ""info"":""" &amp; DE2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/4/1-2026/5/31", "2026/7/18-2026/8/31", "2026/11/1-2026/11/8", "2026/12/21-2026/12/30"], "days":[], "info":"2026通常、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/4/1-2026/5/31", "2026/8/8-2026/8/16"], "days":[], "info":"2026通常、汽船３隻", "data":[</v>
       </c>
       <c r="DJ4" s="8" t="s">
         <v>26</v>
@@ -13582,7 +13579,7 @@
       </c>
       <c r="DR4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DO4 &amp; """, " &amp; DP2 &amp; DQ3 &amp; ", ""info"":""" &amp; DO2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/3/9-2026/3/31", "2026/10/10-2026/10/31"], "days":[], "info":"2026一部変更、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/3/9-2026/3/31"], "days":[], "info":"2026一部変更、汽船３隻", "data":[</v>
       </c>
       <c r="DT4" s="8" t="s">
         <v>26</v>
@@ -13608,7 +13605,7 @@
       </c>
       <c r="EB4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DY4 &amp; """, " &amp; DZ2 &amp; EA3 &amp; ", ""info"":""" &amp; DY2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/7/17", "2026/11/9-2026/12/20"], "days":[], "rinji":"来居欠航時", "info":"2026通常、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/10/10-2026/12/30"], "days":[], "rinji":"来居欠航時", "info":"2026通常、汽船２隻", "data":[</v>
       </c>
       <c r="ED4" s="8" t="s">
         <v>26</v>
@@ -13621,7 +13618,7 @@
       </c>
       <c r="EG4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; ED4 &amp; """, " &amp; EE2 &amp; EF3 &amp; ", ""info"":""" &amp; ED2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/4/1-2026/5/31", "2026/7/18-2026/8/31", "2026/11/1-2026/11/8", "2026/12/21-2026/12/30"], "days":[], "rinji":"来居欠航時", "info":"2026通常、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/4/1-2026/5/31", "2026/8/8-2026/8/16"], "days":[], "rinji":"来居欠航時", "info":"2026通常、汽船３隻", "data":[</v>
       </c>
       <c r="EI4" s="8" t="s">
         <v>26</v>
@@ -13647,7 +13644,7 @@
       </c>
       <c r="EQ4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; EN4 &amp; """, " &amp; EO2 &amp; EP3 &amp; ", ""info"":""" &amp; EN2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/3/9-2026/3/31", "2026/10/10-2026/10/31"], "days":[], "rinji":"来居欠航時", "info":"2026一部変更、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/3/9-2026/3/31"], "days":[], "rinji":"来居欠航時", "info":"2026一部変更、汽船３隻", "data":[</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23296,12 +23293,12 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{D0146144-DB1C-4F97-9719-8B51E4F59984}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{9E9C63D3-FBF0-4976-BCE4-6E50101796A4}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
               <font>
-                <color rgb="00FFFFFF"/>
+                <color rgb="FFFFFFFF"/>
               </font>
               <fill>
                 <patternFill>
@@ -23310,7 +23307,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{691DD0B2-E2C0-4046-8B82-80892632A539}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{7F65E58E-55E7-42FF-AABA-609B5873C520}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>
@@ -30442,12 +30439,12 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{D711BA68-85C4-49DD-AFD9-1BA0F691FD7C}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{F059F3C1-20CD-4D6B-B122-2C8200AC81EC}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
               <font>
-                <color rgb="00FFFFFF"/>
+                <color rgb="FFFFFFFF"/>
               </font>
               <fill>
                 <patternFill>
@@ -30456,7 +30453,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{422C7EA2-99ED-4BDA-BF38-561420AA3B15}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{A14C6024-5FA3-494B-97B6-B2C1DE77BEEC}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>
@@ -37591,12 +37588,12 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{C518B352-A89B-4CFD-8948-F0D8E1949A72}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{6B5D3E22-255E-4041-90ED-32985EB4971B}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
               <font>
-                <color rgb="00FFFFFF"/>
+                <color rgb="FFFFFFFF"/>
               </font>
               <fill>
                 <patternFill>
@@ -37605,7 +37602,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{CD4C7BDB-38BE-405C-9ED3-778E9C70FD49}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{F49F49E2-D0FF-4AB9-AEB0-1FE6E581E19B}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>

</xml_diff>

<commit_message>
2026 Unlimited. Timetable Change Oct 2026. Android Studio Quail -> Rabbit
</commit_message>
<xml_diff>
--- a/設計データ他/設計・設定.xlsx
+++ b/設計データ他/設計・設定.xlsx
@@ -67,16 +67,16 @@
     <t xml:space="preserve">"spans":["2026/12/31-2027/1/3"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2027/1/4-2027/2/28", "2027/6/1-2027/7/17", "2027/11/9-2027/12/20"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2027/1/4-2027/2/28", "2027/6/1-2027/8/7", "2027/8/17-2027/8/31", "2027/11/1-2027/12/30"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2027/4/1-2027/5/31", "2027/7/18-2027/8/31", "2027/11/1-2027/11/8", "2027/12/21-2027/12/30"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2027/4/1-2027/5/31", "2027/8/8-2027/8/16"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2027/3/1-2027/3/8", "2027/9/1-2027/10/9"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2027/3/1-2027/3/8", "2027/9/1-2027/10/31"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2027/3/9-2027/3/31", "2027/10/10-2027/10/31"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2027/3/9-2027/3/31"], "days":[]</t>
   </si>
   <si>
     <t xml:space="preserve">来居欠航時</t>
@@ -169,13 +169,13 @@
     <t xml:space="preserve">"spans":["2025/12/31-2026/1/3"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/10/10-2026/12/30"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/11/1-2026/12/30"], "days":[]</t>
   </si>
   <si>
     <t xml:space="preserve">"spans":["2026/4/1-2026/5/31", "2026/8/8-2026/8/16"], "days":[]</t>
   </si>
   <si>
-    <t xml:space="preserve">"spans":["2026/3/1-2026/3/8", "2026/9/1-2026/10/9"], "days":[]</t>
+    <t xml:space="preserve">"spans":["2026/3/1-2026/3/8", "2026/9/1-2026/10/31"], "days":[]</t>
   </si>
   <si>
     <t xml:space="preserve">"spans":["2026/3/9-2026/3/31"], "days":[]</t>
@@ -784,9 +784,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>696600</xdr:colOff>
+      <xdr:colOff>696240</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>81360</xdr:rowOff>
+      <xdr:rowOff>81000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -796,7 +796,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2207880" y="5153040"/>
-          <a:ext cx="8536320" cy="3199680"/>
+          <a:ext cx="8535960" cy="3199320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -959,9 +959,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>65880</xdr:colOff>
+      <xdr:colOff>65520</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>167040</xdr:rowOff>
+      <xdr:rowOff>166680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -971,7 +971,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="637920"/>
-          <a:ext cx="8602920" cy="628200"/>
+          <a:ext cx="8602560" cy="627840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1061,9 +1061,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>696600</xdr:colOff>
+      <xdr:colOff>696240</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>81360</xdr:rowOff>
+      <xdr:rowOff>81000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1073,7 +1073,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2207880" y="5153040"/>
-          <a:ext cx="8536320" cy="3199680"/>
+          <a:ext cx="8535960" cy="3199320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1264,9 +1264,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>1865880</xdr:colOff>
+      <xdr:colOff>1865520</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>81360</xdr:rowOff>
+      <xdr:rowOff>81000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1276,7 +1276,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2067120" y="4695840"/>
-          <a:ext cx="9955080" cy="2742480"/>
+          <a:ext cx="9954720" cy="2742120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1467,9 +1467,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>1865880</xdr:colOff>
+      <xdr:colOff>1865520</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>81360</xdr:rowOff>
+      <xdr:rowOff>81000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1479,7 +1479,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2067120" y="4695840"/>
-          <a:ext cx="9955080" cy="2056680"/>
+          <a:ext cx="9954720" cy="2056320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="DC4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; CZ4 &amp; """, " &amp; DA2 &amp; DB3 &amp; ", ""info"":""" &amp; CZ2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/1/4-2027/2/28", "2027/6/1-2027/7/17", "2027/11/9-2027/12/20"], "days":[], "info":"2027通常、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/1/4-2027/2/28", "2027/6/1-2027/8/7", "2027/8/17-2027/8/31", "2027/11/1-2027/12/30"], "days":[], "info":"2027通常、汽船２隻", "data":[</v>
       </c>
       <c r="DE4" s="8" t="s">
         <v>26</v>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="DH4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DE4 &amp; """, " &amp; DF2 &amp; DG3 &amp; ", ""info"":""" &amp; DE2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/4/1-2027/5/31", "2027/7/18-2027/8/31", "2027/11/1-2027/11/8", "2027/12/21-2027/12/30"], "days":[], "info":"2027通常、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/4/1-2027/5/31", "2027/8/8-2027/8/16"], "days":[], "info":"2027通常、汽船３隻", "data":[</v>
       </c>
       <c r="DJ4" s="8" t="s">
         <v>26</v>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="DM4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DJ4 &amp; """, " &amp; DK2 &amp; DL3 &amp; ", ""info"":""" &amp; DJ2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/3/1-2027/3/8", "2027/9/1-2027/10/9"], "days":[], "info":"2027一部変更、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/3/1-2027/3/8", "2027/9/1-2027/10/31"], "days":[], "info":"2027一部変更、汽船２隻", "data":[</v>
       </c>
       <c r="DO4" s="8" t="s">
         <v>26</v>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="DR4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DO4 &amp; """, " &amp; DP2 &amp; DQ3 &amp; ", ""info"":""" &amp; DO2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/3/9-2027/3/31", "2027/10/10-2027/10/31"], "days":[], "info":"2027一部変更、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/3/9-2027/3/31"], "days":[], "info":"2027一部変更、汽船３隻", "data":[</v>
       </c>
       <c r="DT4" s="8" t="s">
         <v>26</v>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="EB4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DY4 &amp; """, " &amp; DZ2 &amp; EA3 &amp; ", ""info"":""" &amp; DY2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/1/4-2027/2/28", "2027/6/1-2027/7/17", "2027/11/9-2027/12/20"], "days":[], "rinji":"来居欠航時", "info":"2027通常、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/1/4-2027/2/28", "2027/6/1-2027/8/7", "2027/8/17-2027/8/31", "2027/11/1-2027/12/30"], "days":[], "rinji":"来居欠航時", "info":"2027通常、汽船２隻", "data":[</v>
       </c>
       <c r="ED4" s="8" t="s">
         <v>26</v>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="EG4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; ED4 &amp; """, " &amp; EE2 &amp; EF3 &amp; ", ""info"":""" &amp; ED2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/4/1-2027/5/31", "2027/7/18-2027/8/31", "2027/11/1-2027/11/8", "2027/12/21-2027/12/30"], "days":[], "rinji":"来居欠航時", "info":"2027通常、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/4/1-2027/5/31", "2027/8/8-2027/8/16"], "days":[], "rinji":"来居欠航時", "info":"2027通常、汽船３隻", "data":[</v>
       </c>
       <c r="EI4" s="8" t="s">
         <v>26</v>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="EL4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; EI4 &amp; """, " &amp; EJ2 &amp; EK3 &amp; ", ""info"":""" &amp; EI2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/3/1-2027/3/8", "2027/9/1-2027/10/9"], "days":[], "rinji":"来居欠航時", "info":"2027一部変更、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/3/1-2027/3/8", "2027/9/1-2027/10/31"], "days":[], "rinji":"来居欠航時", "info":"2027一部変更、汽船２隻", "data":[</v>
       </c>
       <c r="EN4" s="8" t="s">
         <v>26</v>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="EQ4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; EN4 &amp; """, " &amp; EO2 &amp; EP3 &amp; ", ""info"":""" &amp; EN2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2027/3/9-2027/3/31", "2027/10/10-2027/10/31"], "days":[], "rinji":"来居欠航時", "info":"2027一部変更、汽船３隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2027/3/9-2027/3/31"], "days":[], "rinji":"来居欠航時", "info":"2027一部変更、汽船３隻", "data":[</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12484,7 +12484,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{E2BAB997-E02C-43CF-A2D0-2D3DEC14A97A}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{E971D15E-37B7-4B70-99C9-FCE33E80A0E6}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
@@ -12498,7 +12498,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{DA90B542-3FD6-49C0-B339-2F7653A86F78}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{DDFC82E7-C1E3-417D-B471-10F0559D41FD}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>
@@ -12507,7 +12507,59 @@
               </font>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>1:1048576</xm:sqref>
+          <xm:sqref>1:1 3:1048576 DQ2:ED2 EP2:XFD2 EF2:EN2 DG2:DO2 A2:DE2</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{4378DC4D-D336-4F50-B8EC-578A7C315BD2}">
+            <xm:f>NOT(ISERROR(SEARCH($A$1-2,DF2)))</xm:f>
+            <xm:f>$A$1-2</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FFFFFFFF"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{3BFE6B65-21B6-4FE4-ABCA-B8A74971EF19}">
+            <xm:f>NOT(ISERROR(SEARCH($A$1-1,DF2)))</xm:f>
+            <xm:f>$A$1-1</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FFC00000"/>
+              </font>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>EE2 DF2</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="6" operator="containsText" id="{D8D081E8-C69B-4BD8-AE79-4B48A8401B32}">
+            <xm:f>NOT(ISERROR(SEARCH($A$1-2,DP2)))</xm:f>
+            <xm:f>$A$1-2</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FFFFFFFF"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="7" operator="containsText" id="{A69A15FE-5656-4DE4-BE3D-A7D831167255}">
+            <xm:f>NOT(ISERROR(SEARCH($A$1-1,DP2)))</xm:f>
+            <xm:f>$A$1-1</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FFC00000"/>
+              </font>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>EO2 DP2</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -13540,7 +13592,7 @@
       </c>
       <c r="DC4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; CZ4 &amp; """, " &amp; DA2 &amp; DB3 &amp; ", ""info"":""" &amp; CZ2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/10/10-2026/12/30"], "days":[], "info":"2026通常、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/11/1-2026/12/30"], "days":[], "info":"2026通常、汽船２隻", "data":[</v>
       </c>
       <c r="DE4" s="8" t="s">
         <v>26</v>
@@ -13566,7 +13618,7 @@
       </c>
       <c r="DM4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DJ4 &amp; """, " &amp; DK2 &amp; DL3 &amp; ", ""info"":""" &amp; DJ2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/3/1-2026/3/8", "2026/9/1-2026/10/9"], "days":[], "info":"2026一部変更、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/3/1-2026/3/8", "2026/9/1-2026/10/31"], "days":[], "info":"2026一部変更、汽船２隻", "data":[</v>
       </c>
       <c r="DO4" s="8" t="s">
         <v>26</v>
@@ -13605,7 +13657,7 @@
       </c>
       <c r="EB4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; DY4 &amp; """, " &amp; DZ2 &amp; EA3 &amp; ", ""info"":""" &amp; DY2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/10/10-2026/12/30"], "days":[], "rinji":"来居欠航時", "info":"2026通常、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/1/4-2026/2/28", "2026/6/1-2026/8/7", "2026/8/17-2026/8/31", "2026/11/1-2026/12/30"], "days":[], "rinji":"来居欠航時", "info":"2026通常、汽船２隻", "data":[</v>
       </c>
       <c r="ED4" s="8" t="s">
         <v>26</v>
@@ -13631,7 +13683,7 @@
       </c>
       <c r="EL4" s="8" t="str">
         <f aca="false">"{""ship"":""" &amp; EI4 &amp; """, " &amp; EJ2 &amp; EK3 &amp; ", ""info"":""" &amp; EI2 &amp; """, ""data"":["</f>
-        <v>{"ship":"いそかぜ", "spans":["2026/3/1-2026/3/8", "2026/9/1-2026/10/9"], "days":[], "rinji":"来居欠航時", "info":"2026一部変更、汽船２隻", "data":[</v>
+        <v>{"ship":"いそかぜ", "spans":["2026/3/1-2026/3/8", "2026/9/1-2026/10/31"], "days":[], "rinji":"来居欠航時", "info":"2026一部変更、汽船２隻", "data":[</v>
       </c>
       <c r="EN4" s="8" t="s">
         <v>26</v>
@@ -23293,7 +23345,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{9E9C63D3-FBF0-4976-BCE4-6E50101796A4}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{2210AAB7-A465-4056-A715-B4E28E50D618}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
@@ -23307,7 +23359,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{7F65E58E-55E7-42FF-AABA-609B5873C520}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{3EB16840-92EA-4E15-8B60-D43FB612309C}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>
@@ -23316,7 +23368,33 @@
               </font>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>1:1048576</xm:sqref>
+          <xm:sqref>1:3 34:1048576 A4:EF33 EH4:XFD33</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{93157DC2-192B-4785-A466-7B58E5BC10AD}">
+            <xm:f>NOT(ISERROR(SEARCH($A$1-2,EG4)))</xm:f>
+            <xm:f>$A$1-2</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FFFFFFFF"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{1D904E96-ADA4-475E-94B8-9EB94912C5F6}">
+            <xm:f>NOT(ISERROR(SEARCH($A$1-1,EG4)))</xm:f>
+            <xm:f>$A$1-1</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FFC00000"/>
+              </font>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>EG4:EG33</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -30439,7 +30517,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{F059F3C1-20CD-4D6B-B122-2C8200AC81EC}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{87219DB0-A840-47F4-85F9-148AC2531E41}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
@@ -30453,7 +30531,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{A14C6024-5FA3-494B-97B6-B2C1DE77BEEC}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{EBB71070-BCFC-4C33-B9FE-A319D07240F7}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>
@@ -37588,7 +37666,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{6B5D3E22-255E-4041-90ED-32985EB4971B}">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{3E76DD84-E280-4163-BBB1-F7A729AB8FDF}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-2,A1)))</xm:f>
             <xm:f>$A$1-2</xm:f>
             <x14:dxf>
@@ -37602,7 +37680,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{F49F49E2-D0FF-4AB9-AEB0-1FE6E581E19B}">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{758B4297-8D80-46C6-9F60-F3D8321029DE}">
             <xm:f>NOT(ISERROR(SEARCH($A$1-1,A1)))</xm:f>
             <xm:f>$A$1-1</xm:f>
             <x14:dxf>

</xml_diff>